<commit_message>
Update link in books.md to reference books.xlsx
</commit_message>
<xml_diff>
--- a/books.xlsx
+++ b/books.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="book_I_own" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">book_I_own!$A$1:$G$61</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="107">
   <si>
     <t>Title</t>
   </si>
@@ -50,36 +53,45 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>2024 Backend Roadmap</t>
+    <t>2020-Scrum-Guide-Tamil-3.0</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>2020-Scrum-Guide-US</t>
+  </si>
+  <si>
+    <t>2024 Backend Roadmap - Light</t>
   </si>
   <si>
     <t>Roadmap</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Backend</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>By web dev simplified</t>
   </si>
   <si>
-    <t>2024 Frontend Roadmap</t>
+    <t>2024 Frontend Roadmap - Light</t>
   </si>
   <si>
     <t>Frontend</t>
   </si>
   <si>
-    <t>Blender by Wiki books</t>
+    <t>Blender Doc by Wikipedia</t>
   </si>
   <si>
     <t>Blender</t>
   </si>
   <si>
+    <t>Byte Of Python</t>
+  </si>
+  <si>
     <t>Clean Architectures in Python E2</t>
   </si>
   <si>
@@ -101,6 +113,12 @@
     <t>Packt free book</t>
   </si>
   <si>
+    <t>Communication_Beginnings_An_Introductory_Listening_and_Speaking</t>
+  </si>
+  <si>
+    <t>CSCI 3410 - Database Systems (Lecture Notes)</t>
+  </si>
+  <si>
     <t>CSS Notes</t>
   </si>
   <si>
@@ -122,6 +140,12 @@
     <t>Database Systems for Management E3</t>
   </si>
   <si>
+    <t>Django 5 By Example</t>
+  </si>
+  <si>
+    <t>Django 5 By Example Color Images</t>
+  </si>
+  <si>
     <t>Docker Cookbook 2E</t>
   </si>
   <si>
@@ -134,6 +158,9 @@
     <t>Not Yet</t>
   </si>
   <si>
+    <t>Docker roadmap</t>
+  </si>
+  <si>
     <t>Eloquent JavaScript E4</t>
   </si>
   <si>
@@ -146,6 +173,15 @@
     <t>Evidence-based Software Engineering</t>
   </si>
   <si>
+    <t>For Style Inspire 1</t>
+  </si>
+  <si>
+    <t>For Style Inspire 2</t>
+  </si>
+  <si>
+    <t>Front-end Developer Handbook 2019</t>
+  </si>
+  <si>
     <t>Git Notes</t>
   </si>
   <si>
@@ -167,6 +203,12 @@
     <t>HTML5 Notes</t>
   </si>
   <si>
+    <t>IBM DevOps for Dummies E3</t>
+  </si>
+  <si>
+    <t>IBM_Database Fundamentals E1_2010</t>
+  </si>
+  <si>
     <t>Introduction to Networking</t>
   </si>
   <si>
@@ -182,6 +224,18 @@
     <t>LaTeX</t>
   </si>
   <si>
+    <t>Learn Object Oriented Thinking and Programming Java</t>
+  </si>
+  <si>
+    <t>Learning MongoDB</t>
+  </si>
+  <si>
+    <t>Learning MySQL</t>
+  </si>
+  <si>
+    <t>Learning MySQL By Example</t>
+  </si>
+  <si>
     <t>Learning Patterns</t>
   </si>
   <si>
@@ -212,6 +266,9 @@
     <t>RDBMS</t>
   </si>
   <si>
+    <t>Postgre The First Experience</t>
+  </si>
+  <si>
     <t>PostgreSQL Notes</t>
   </si>
   <si>
@@ -227,12 +284,24 @@
     <t>Python Notes</t>
   </si>
   <si>
+    <t>Python Programming Modular Approach</t>
+  </si>
+  <si>
+    <t>Python Succinctly</t>
+  </si>
+  <si>
+    <t>Quantum Computing for the Quantum Curious</t>
+  </si>
+  <si>
     <t>ReactJS Notes</t>
   </si>
   <si>
     <t>ReactJS</t>
   </si>
   <si>
+    <t>Readings in Database Systems E5</t>
+  </si>
+  <si>
     <t>Responsive Web Design with HTML5 and CSS3 2E</t>
   </si>
   <si>
@@ -273,6 +342,9 @@
   </si>
   <si>
     <t>TypeScript</t>
+  </si>
+  <si>
+    <t>Understanding the DOM</t>
   </si>
   <si>
     <t>Visual Studio Code Keyboard Shortcuts</t>
@@ -291,7 +363,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,13 +373,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -762,154 +827,157 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -962,6 +1030,18 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1229,7 +1309,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="48.4285714285714" customWidth="1"/>
@@ -1272,177 +1352,177 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" t="s">
         <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G9" t="s">
         <v>26</v>
@@ -1450,666 +1530,1207 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G11" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="F12" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G15" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="D17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G17" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="D18" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="F18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G18" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G19" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="F20" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="G20" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G22" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="D23" t="s">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G23" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G24" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="D25" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G25" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G26" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G27" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="D28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="D29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E29" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F29" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="G29" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="D30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G30" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D31" t="s">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="E31" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="D32" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E32" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F32" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G32" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G33" t="s">
-        <v>74</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G34" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G35" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C36" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G36" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" t="s">
+        <v>69</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" t="s">
+        <v>8</v>
+      </c>
+      <c r="G38" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>9</v>
+      </c>
+      <c r="F39" t="s">
+        <v>8</v>
+      </c>
+      <c r="G39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" t="s">
+        <v>74</v>
+      </c>
+      <c r="E40" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" t="s">
+        <v>8</v>
+      </c>
+      <c r="G40" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" t="s">
+        <v>8</v>
+      </c>
+      <c r="G41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s">
+        <v>8</v>
+      </c>
+      <c r="G42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" t="s">
+        <v>79</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
         <v>80</v>
       </c>
-      <c r="B37" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="D43" t="s">
+        <v>77</v>
+      </c>
+      <c r="E43" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" t="s">
+        <v>8</v>
+      </c>
+      <c r="G43" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
         <v>81</v>
       </c>
-      <c r="D37" t="s">
-        <v>9</v>
-      </c>
-      <c r="E37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" t="s">
-        <v>9</v>
-      </c>
-      <c r="G37" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" t="s">
+      <c r="B44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
         <v>82</v>
       </c>
-      <c r="B38" t="s">
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" t="s">
+        <v>8</v>
+      </c>
+      <c r="G44" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
         <v>83</v>
       </c>
-      <c r="C38" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" t="s">
-        <v>9</v>
-      </c>
-      <c r="E38" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" t="s">
-        <v>9</v>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>9</v>
+      </c>
+      <c r="F45" t="s">
+        <v>8</v>
+      </c>
+      <c r="G45" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" t="s">
+        <v>8</v>
+      </c>
+      <c r="G46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" t="s">
+        <v>9</v>
+      </c>
+      <c r="F47" t="s">
+        <v>8</v>
+      </c>
+      <c r="G47" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" t="s">
+        <v>9</v>
+      </c>
+      <c r="F48" t="s">
+        <v>8</v>
+      </c>
+      <c r="G48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>88</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>9</v>
+      </c>
+      <c r="F49" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
+        <v>89</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" t="s">
+        <v>9</v>
+      </c>
+      <c r="F50" t="s">
+        <v>8</v>
+      </c>
+      <c r="G50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>53</v>
+      </c>
+      <c r="D51" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" t="s">
+        <v>9</v>
+      </c>
+      <c r="F51" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>92</v>
+      </c>
+      <c r="D52" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" t="s">
+        <v>8</v>
+      </c>
+      <c r="G52" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" t="s">
+        <v>9</v>
+      </c>
+      <c r="F53" t="s">
+        <v>8</v>
+      </c>
+      <c r="G53" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" t="s">
+        <v>94</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
+        <v>60</v>
+      </c>
+      <c r="E54" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" t="s">
+        <v>8</v>
+      </c>
+      <c r="G54" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" t="s">
+        <v>8</v>
+      </c>
+      <c r="G55" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" t="s">
+        <v>98</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" t="s">
+        <v>9</v>
+      </c>
+      <c r="F56" t="s">
+        <v>8</v>
+      </c>
+      <c r="G56" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" t="s">
+        <v>100</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" t="s">
+        <v>9</v>
+      </c>
+      <c r="F57" t="s">
+        <v>8</v>
+      </c>
+      <c r="G57" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" t="s">
+        <v>102</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" t="s">
+        <v>103</v>
+      </c>
+      <c r="D59" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" t="s">
+        <v>8</v>
+      </c>
+      <c r="G59" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" t="s">
+        <v>8</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" t="s">
+        <v>9</v>
+      </c>
+      <c r="F60" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" t="s">
+        <v>105</v>
+      </c>
+      <c r="B61" t="s">
+        <v>106</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" t="s">
+        <v>9</v>
+      </c>
+      <c r="F61" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G61" etc:filterBottomFollowUsedRange="0">
+    <sortState ref="A2:G61">
+      <sortCondition ref="A1"/>
+    </sortState>
+    <extLst/>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:A61">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>

</xml_diff>